<commit_message>
Update EOD data and reports for 20 Feb 2026 with final closing prices
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260220.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260220.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.687</v>
+        <v>1.695</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.007</v>
+        <v>0.015</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.42%</t>
+          <t>0.89%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>258416.35</v>
+        <v>259641.8</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>1072.27</v>
+        <v>2297.72</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1.35</v>
+        <v>1.352</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.02</v>
+        <v>-0.018</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-1.46%</t>
+          <t>-1.31%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>94500</v>
+        <v>94640</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-1400</v>
+        <v>-1260</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1.595</v>
+        <v>1.59</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.025</v>
+        <v>0.02</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.59%</t>
+          <t>1.27%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>57458</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>91645.50999999999</v>
+        <v>91358.22</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>1436.45</v>
+        <v>1149.16</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>53.77</v>
+        <v>53.745</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.54</v>
+        <v>0.515</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>0.97%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>16361</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>879730.97</v>
+        <v>879321.9399999999</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>8834.940000000001</v>
+        <v>8425.92</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>178.08</v>
+        <v>177.99</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.11</v>
+        <v>-0.2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>-0.11%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -731,24 +731,24 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0.205</v>
+        <v>0.21</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-0.015</v>
+        <v>-0.01</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-6.82%</t>
+          <t>-4.55%</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>1929.46</v>
+        <v>1976.52</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>-141.18</v>
+        <v>-94.12</v>
       </c>
     </row>
     <row r="14">
@@ -785,14 +785,14 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>42.08</v>
+        <v>42.07</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.45%</t>
+          <t>0.43%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
@@ -812,24 +812,24 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>27.14</v>
+        <v>27.145</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.04</v>
+        <v>0.045</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.15%</t>
+          <t>0.17%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>34956.32</v>
+        <v>34962.76</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>51.52</v>
+        <v>57.96</v>
       </c>
     </row>
     <row r="17">
@@ -843,10 +843,10 @@
       <c r="D17" s="5" t="inlineStr"/>
       <c r="E17" s="7" t="inlineStr"/>
       <c r="F17" s="8" t="n">
-        <v>1375957.24</v>
+        <v>1376679.87</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>9804</v>
+        <v>10526.63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add plot_portfolio_value.py and update data/reports through 2026-04-17
Add total portfolio value chart script, update DailyData.csv with
trading data through Apr 17, regenerate all ticker charts, and add
daily reports from Feb 23 to Apr 17.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260220.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260220.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.695</v>
+        <v>1.685</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.015</v>
+        <v>0.005</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.89%</t>
+          <t>0.30%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>259641.8</v>
+        <v>258109.99</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>2297.72</v>
+        <v>765.91</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1.352</v>
+        <v>1.36</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.018</v>
+        <v>-0.01</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-1.31%</t>
+          <t>-0.73%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>94640</v>
+        <v>95200</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-1260</v>
+        <v>-700</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1.59</v>
+        <v>1.585</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.02</v>
+        <v>0.015</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.27%</t>
+          <t>0.96%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>57458</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>91358.22</v>
+        <v>91070.92999999999</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>1149.16</v>
+        <v>861.87</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>53.745</v>
+        <v>53.33</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.515</v>
+        <v>0.1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.97%</t>
+          <t>0.19%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>16361</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>879321.9399999999</v>
+        <v>872532.13</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>8425.92</v>
+        <v>1636.1</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>177.99</v>
+        <v>179.67</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.2</v>
+        <v>1.48</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.11%</t>
+          <t>0.83%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.465</v>
+        <v>0.495</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-0.015</v>
+        <v>0.015</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-3.12%</t>
+          <t>3.13%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>4650</v>
+        <v>4950</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>-150</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>33.33%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>700000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>2100</v>
+        <v>2800</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0</v>
+        <v>700</v>
       </c>
     </row>
     <row r="13">
@@ -731,24 +731,24 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0.21</v>
+        <v>0.225</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-4.55%</t>
+          <t>2.27%</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>1976.52</v>
+        <v>2117.7</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>-94.12</v>
+        <v>47.06</v>
       </c>
     </row>
     <row r="14">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.17</v>
+        <v>0.175</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>2.94%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>1020</v>
+        <v>1050</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15">
@@ -785,14 +785,14 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>42.07</v>
+        <v>42.54</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.18</v>
+        <v>0.65</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>1.55%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
@@ -812,24 +812,24 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>27.145</v>
+        <v>27.43</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.045</v>
+        <v>0.33</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.17%</t>
+          <t>1.22%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>34962.76</v>
+        <v>35329.84</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>57.96</v>
+        <v>425.04</v>
       </c>
     </row>
     <row r="17">
@@ -843,10 +843,10 @@
       <c r="D17" s="5" t="inlineStr"/>
       <c r="E17" s="7" t="inlineStr"/>
       <c r="F17" s="8" t="n">
-        <v>1376679.87</v>
+        <v>1370169.21</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>10526.63</v>
+        <v>4015.98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>